<commit_message>
before add ablation experiment of CA and CutMixand random seed.
</commit_message>
<xml_diff>
--- a/Ablation experiment.xlsx
+++ b/Ablation experiment.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/haochen/Documents/Development/bright-cmca/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{412A03C6-0FC6-1945-982B-3ACEA97344C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C623E984-AF38-0240-9E36-C4F2E280F6EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4340" yWindow="760" windowWidth="30220" windowHeight="20000" firstSheet="1" activeTab="7" xr2:uid="{79C5FF15-FE7B-B844-917A-3EB10CF0BE82}"/>
+    <workbookView xWindow="4340" yWindow="760" windowWidth="30220" windowHeight="20000" firstSheet="6" activeTab="13" xr2:uid="{79C5FF15-FE7B-B844-917A-3EB10CF0BE82}"/>
   </bookViews>
   <sheets>
     <sheet name="Overall" sheetId="7" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="96">
   <si>
     <t>Method</t>
   </si>
@@ -169,9 +169,6 @@
   </si>
   <si>
     <t>SiamAttnUNet + CMCA + CutMix 0.25</t>
-  </si>
-  <si>
-    <t>SiamAttnUNet + CMCA + CutMix 0.30</t>
   </si>
   <si>
     <t>SiamAttnUNet + CutMix 0.25</t>
@@ -210,10 +207,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>SiamAttnUNet + CutMix 0.30</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>DamageFormer + CutMix 0.25</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -359,6 +352,14 @@
   </si>
   <si>
     <t>SiamAttnUNet + CMCA + CutMix 0.3</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>SiamAttnUNet</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Best</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -393,14 +394,6 @@
     </font>
     <font>
       <sz val="12"/>
-      <color rgb="FF333333"/>
-      <name val="等线"/>
-      <family val="4"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="等线"/>
       <family val="4"/>
@@ -416,8 +409,16 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <family val="4"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -436,6 +437,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -451,7 +458,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -464,9 +471,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -476,7 +480,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -494,14 +498,23 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1167,28 +1180,28 @@
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="5">
+      <c r="B2" s="4">
         <v>88.32</v>
       </c>
-      <c r="C2" s="5">
+      <c r="C2" s="4">
         <v>70.91</v>
       </c>
-      <c r="D2" s="5">
+      <c r="D2" s="4">
         <v>95.52</v>
       </c>
-      <c r="E2" s="5">
+      <c r="E2" s="4">
         <v>64.739999999999995</v>
       </c>
-      <c r="F2" s="5">
+      <c r="F2" s="4">
         <v>96.28</v>
       </c>
-      <c r="G2" s="5">
+      <c r="G2" s="4">
         <v>71.62</v>
       </c>
-      <c r="H2" s="5">
+      <c r="H2" s="4">
         <v>37.479999999999997</v>
       </c>
-      <c r="I2" s="5">
+      <c r="I2" s="4">
         <v>53.59</v>
       </c>
     </row>
@@ -1196,57 +1209,57 @@
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="5">
+      <c r="B3" s="4">
         <v>88.65</v>
       </c>
-      <c r="C3" s="5">
+      <c r="C3" s="4">
         <v>70.180000000000007</v>
       </c>
-      <c r="D3" s="5">
+      <c r="D3" s="4">
         <v>95.54</v>
       </c>
-      <c r="E3" s="5">
+      <c r="E3" s="4">
         <v>64.44</v>
       </c>
-      <c r="F3" s="5">
+      <c r="F3" s="4">
         <v>96.28</v>
       </c>
-      <c r="G3" s="5">
+      <c r="G3" s="4">
         <v>72.36</v>
       </c>
-      <c r="H3" s="5">
+      <c r="H3" s="4">
         <v>36.270000000000003</v>
       </c>
-      <c r="I3" s="5">
+      <c r="I3" s="4">
         <v>52.84</v>
       </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="B4" s="5">
+        <v>52</v>
+      </c>
+      <c r="B4" s="4">
         <v>88.07</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="4">
         <v>70.89</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="4">
         <v>95.48</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="4">
         <v>64.459999999999994</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="4">
         <v>96.22</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="4">
         <v>71.430000000000007</v>
       </c>
-      <c r="H4" s="5">
+      <c r="H4" s="4">
         <v>38.049999999999997</v>
       </c>
-      <c r="I4" s="5">
+      <c r="I4" s="4">
         <v>52.15</v>
       </c>
     </row>
@@ -1254,28 +1267,28 @@
       <c r="A5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="5">
+      <c r="B5" s="4">
         <v>88.68</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="5">
         <v>72.650000000000006</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="4">
         <v>95.59</v>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="4">
         <v>65.39</v>
       </c>
-      <c r="F5" s="5">
+      <c r="F5" s="4">
         <v>96.29</v>
       </c>
-      <c r="G5" s="5">
+      <c r="G5" s="4">
         <v>72.790000000000006</v>
       </c>
-      <c r="H5" s="5">
+      <c r="H5" s="4">
         <v>39.299999999999997</v>
       </c>
-      <c r="I5" s="5">
+      <c r="I5" s="4">
         <v>53.2</v>
       </c>
     </row>
@@ -1283,28 +1296,28 @@
       <c r="A6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="5">
+      <c r="B6" s="4">
         <v>89.09</v>
       </c>
-      <c r="C6" s="5">
+      <c r="C6" s="4">
         <v>72.03</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="5">
         <v>95.82</v>
       </c>
-      <c r="E6" s="5">
+      <c r="E6" s="4">
         <v>66.069999999999993</v>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="5">
         <v>96.52</v>
       </c>
-      <c r="G6" s="5">
+      <c r="G6" s="4">
         <v>73.290000000000006</v>
       </c>
-      <c r="H6" s="6">
+      <c r="H6" s="5">
         <v>40.53</v>
       </c>
-      <c r="I6" s="5">
+      <c r="I6" s="4">
         <v>53.93</v>
       </c>
     </row>
@@ -1312,28 +1325,28 @@
       <c r="A7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="6">
+      <c r="B7" s="5">
         <v>89.18</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="4">
         <v>72.430000000000007</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="4">
         <v>95.81</v>
       </c>
-      <c r="E7" s="6">
+      <c r="E7" s="5">
         <v>66.16</v>
       </c>
-      <c r="F7" s="5">
+      <c r="F7" s="4">
         <v>96.5</v>
       </c>
-      <c r="G7" s="6">
+      <c r="G7" s="5">
         <v>73.58</v>
       </c>
-      <c r="H7" s="5">
+      <c r="H7" s="4">
         <v>39.08</v>
       </c>
-      <c r="I7" s="6">
+      <c r="I7" s="5">
         <v>55.49</v>
       </c>
     </row>
@@ -1341,57 +1354,57 @@
       <c r="A8" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="7">
+      <c r="B8" s="6">
         <v>89.88</v>
       </c>
-      <c r="C8" s="7">
+      <c r="C8" s="6">
         <v>72.61</v>
       </c>
-      <c r="D8" s="7">
+      <c r="D8" s="6">
         <v>96</v>
       </c>
-      <c r="E8" s="7">
+      <c r="E8" s="6">
         <v>66.84</v>
       </c>
-      <c r="F8" s="7">
+      <c r="F8" s="6">
         <v>96.7</v>
       </c>
-      <c r="G8" s="7">
+      <c r="G8" s="6">
         <v>74.62</v>
       </c>
-      <c r="H8" s="7">
+      <c r="H8" s="6">
         <v>39.97</v>
       </c>
-      <c r="I8" s="7">
+      <c r="I8" s="6">
         <v>56.06</v>
       </c>
     </row>
     <row r="9" spans="1:9">
       <c r="A9" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="B9" s="8">
+        <v>51</v>
+      </c>
+      <c r="B9" s="7">
         <v>89.91</v>
       </c>
-      <c r="C9" s="8">
+      <c r="C9" s="7">
         <v>72.25</v>
       </c>
-      <c r="D9" s="8">
+      <c r="D9" s="7">
         <v>96.04</v>
       </c>
-      <c r="E9" s="8">
+      <c r="E9" s="7">
         <v>66.790000000000006</v>
       </c>
-      <c r="F9" s="8">
+      <c r="F9" s="7">
         <v>96.75</v>
       </c>
-      <c r="G9" s="8">
+      <c r="G9" s="7">
         <v>74.680000000000007</v>
       </c>
-      <c r="H9" s="8">
+      <c r="H9" s="7">
         <v>39.03</v>
       </c>
-      <c r="I9" s="8">
+      <c r="I9" s="7">
         <v>56.7</v>
       </c>
     </row>
@@ -1399,28 +1412,28 @@
       <c r="A10" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B10" s="7">
+      <c r="B10" s="6">
         <v>89.94</v>
       </c>
-      <c r="C10" s="7">
+      <c r="C10" s="6">
         <v>73.05</v>
       </c>
-      <c r="D10" s="9">
+      <c r="D10" s="8">
         <v>96.09</v>
       </c>
-      <c r="E10" s="9">
+      <c r="E10" s="8">
         <v>67.2</v>
       </c>
-      <c r="F10" s="9">
+      <c r="F10" s="8">
         <v>96.77</v>
       </c>
-      <c r="G10" s="9">
+      <c r="G10" s="8">
         <v>74.94</v>
       </c>
-      <c r="H10" s="9">
+      <c r="H10" s="8">
         <v>41.4</v>
       </c>
-      <c r="I10" s="7">
+      <c r="I10" s="6">
         <v>55.7</v>
       </c>
     </row>
@@ -1428,28 +1441,28 @@
       <c r="A11" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="7">
+      <c r="B11" s="6">
         <v>89.9</v>
       </c>
-      <c r="C11" s="7">
+      <c r="C11" s="6">
         <v>71.959999999999994</v>
       </c>
-      <c r="D11" s="7">
+      <c r="D11" s="6">
         <v>95.97</v>
       </c>
-      <c r="E11" s="7">
+      <c r="E11" s="6">
         <v>66.55</v>
       </c>
-      <c r="F11" s="7">
+      <c r="F11" s="6">
         <v>96.72</v>
       </c>
-      <c r="G11" s="7">
+      <c r="G11" s="6">
         <v>74.349999999999994</v>
       </c>
-      <c r="H11" s="7">
+      <c r="H11" s="6">
         <v>38.61</v>
       </c>
-      <c r="I11" s="7">
+      <c r="I11" s="6">
         <v>56.53</v>
       </c>
     </row>
@@ -1457,28 +1470,28 @@
       <c r="A12" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="9">
+      <c r="B12" s="8">
         <v>90</v>
       </c>
-      <c r="C12" s="7">
+      <c r="C12" s="6">
         <v>72.39</v>
       </c>
-      <c r="D12" s="7">
+      <c r="D12" s="6">
         <v>96</v>
       </c>
-      <c r="E12" s="7">
+      <c r="E12" s="6">
         <v>66.650000000000006</v>
       </c>
-      <c r="F12" s="7">
+      <c r="F12" s="6">
         <v>96.74</v>
       </c>
-      <c r="G12" s="7">
+      <c r="G12" s="6">
         <v>74.62</v>
       </c>
-      <c r="H12" s="7">
+      <c r="H12" s="6">
         <v>39.49</v>
       </c>
-      <c r="I12" s="7">
+      <c r="I12" s="6">
         <v>55.74</v>
       </c>
     </row>
@@ -1486,382 +1499,382 @@
       <c r="A13" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="7">
+      <c r="B13" s="6">
         <v>89.91</v>
       </c>
-      <c r="C13" s="9">
+      <c r="C13" s="8">
         <v>73.069999999999993</v>
       </c>
-      <c r="D13" s="7">
+      <c r="D13" s="6">
         <v>96</v>
       </c>
-      <c r="E13" s="7">
+      <c r="E13" s="6">
         <v>67.14</v>
       </c>
-      <c r="F13" s="7">
+      <c r="F13" s="6">
         <v>96.71</v>
       </c>
-      <c r="G13" s="7">
+      <c r="G13" s="6">
         <v>74.540000000000006</v>
       </c>
-      <c r="H13" s="7">
+      <c r="H13" s="6">
         <v>40.17</v>
       </c>
-      <c r="I13" s="9">
+      <c r="I13" s="8">
         <v>57.12</v>
       </c>
     </row>
     <row r="14" spans="1:9">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="B14" s="5">
+      <c r="B14" s="16">
         <v>88.26</v>
       </c>
-      <c r="C14" s="5">
+      <c r="C14" s="16">
         <v>71.790000000000006</v>
       </c>
-      <c r="D14" s="5">
+      <c r="D14" s="16">
         <v>95.51</v>
       </c>
-      <c r="E14" s="5">
+      <c r="E14" s="16">
         <v>65.03</v>
       </c>
-      <c r="F14" s="5">
+      <c r="F14" s="16">
         <v>96.21</v>
       </c>
-      <c r="G14" s="5">
+      <c r="G14" s="16">
         <v>72.06</v>
       </c>
-      <c r="H14" s="5">
+      <c r="H14" s="16">
         <v>38.24</v>
       </c>
-      <c r="I14" s="5">
+      <c r="I14" s="16">
         <v>53.6</v>
       </c>
     </row>
     <row r="15" spans="1:9">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="B15" s="5">
+      <c r="B15" s="16">
         <v>88.03</v>
       </c>
-      <c r="C15" s="5">
+      <c r="C15" s="16">
         <v>71.989999999999995</v>
       </c>
-      <c r="D15" s="5">
+      <c r="D15" s="16">
         <v>95.53</v>
       </c>
-      <c r="E15" s="5">
+      <c r="E15" s="16">
         <v>65.27</v>
       </c>
-      <c r="F15" s="5">
+      <c r="F15" s="16">
         <v>96.15</v>
       </c>
-      <c r="G15" s="5">
+      <c r="G15" s="16">
         <v>72</v>
       </c>
-      <c r="H15" s="5">
+      <c r="H15" s="16">
         <v>39.08</v>
       </c>
-      <c r="I15" s="5">
+      <c r="I15" s="16">
         <v>53.83</v>
       </c>
     </row>
     <row r="16" spans="1:9">
-      <c r="A16" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="B16" s="5">
+      <c r="A16" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="B16" s="16">
         <v>87.92</v>
       </c>
-      <c r="C16" s="5">
+      <c r="C16" s="16">
         <v>71.849999999999994</v>
       </c>
-      <c r="D16" s="5">
+      <c r="D16" s="16">
         <v>95.49</v>
       </c>
-      <c r="E16" s="5">
+      <c r="E16" s="16">
         <v>65.28</v>
       </c>
-      <c r="F16" s="5">
+      <c r="F16" s="16">
         <v>96.11</v>
       </c>
-      <c r="G16" s="5">
+      <c r="G16" s="16">
         <v>71.95</v>
       </c>
-      <c r="H16" s="5">
+      <c r="H16" s="16">
         <v>37.450000000000003</v>
       </c>
-      <c r="I16" s="5">
+      <c r="I16" s="16">
         <v>55.62</v>
       </c>
     </row>
     <row r="17" spans="1:9">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="B17" s="5">
-        <v>88.6</v>
-      </c>
-      <c r="C17" s="5">
-        <v>71.510000000000005</v>
-      </c>
-      <c r="D17" s="5">
-        <v>95.56</v>
-      </c>
-      <c r="E17" s="5">
-        <v>64.81</v>
-      </c>
-      <c r="F17" s="5">
-        <v>96.32</v>
-      </c>
-      <c r="G17" s="5">
-        <v>72.12</v>
-      </c>
-      <c r="H17" s="5">
-        <v>38.81</v>
-      </c>
-      <c r="I17" s="5">
-        <v>52.01</v>
+      <c r="B17" s="16">
+        <v>88.08</v>
+      </c>
+      <c r="C17" s="16">
+        <v>72.150000000000006</v>
+      </c>
+      <c r="D17" s="16">
+        <v>95.49</v>
+      </c>
+      <c r="E17" s="16">
+        <v>65.05</v>
+      </c>
+      <c r="F17" s="16">
+        <v>96.19</v>
+      </c>
+      <c r="G17" s="16">
+        <v>71.67</v>
+      </c>
+      <c r="H17" s="16">
+        <v>39.5</v>
+      </c>
+      <c r="I17" s="16">
+        <v>52.84</v>
       </c>
     </row>
     <row r="18" spans="1:9">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="B18" s="5">
-        <v>88.21</v>
-      </c>
-      <c r="C18" s="5">
-        <v>71.59</v>
-      </c>
-      <c r="D18" s="5">
-        <v>95.61</v>
-      </c>
-      <c r="E18" s="5">
-        <v>65.709999999999994</v>
-      </c>
-      <c r="F18" s="5">
-        <v>96.26</v>
-      </c>
-      <c r="G18" s="5">
-        <v>72.150000000000006</v>
-      </c>
-      <c r="H18" s="5">
-        <v>37.56</v>
-      </c>
-      <c r="I18" s="6">
-        <v>56.86</v>
+      <c r="B18" s="17">
+        <v>88.44</v>
+      </c>
+      <c r="C18" s="17">
+        <v>72.67</v>
+      </c>
+      <c r="D18" s="17">
+        <v>95.67</v>
+      </c>
+      <c r="E18" s="17">
+        <v>66.28</v>
+      </c>
+      <c r="F18" s="17">
+        <v>96.33</v>
+      </c>
+      <c r="G18" s="17">
+        <v>72.55</v>
+      </c>
+      <c r="H18" s="16">
+        <v>38.94</v>
+      </c>
+      <c r="I18" s="17">
+        <v>57.3</v>
       </c>
     </row>
     <row r="19" spans="1:9">
-      <c r="A19" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="B19" s="6">
-        <v>88.77</v>
-      </c>
-      <c r="C19" s="6">
-        <v>72.88</v>
-      </c>
-      <c r="D19" s="6">
-        <v>95.71</v>
-      </c>
-      <c r="E19" s="6">
-        <v>66.260000000000005</v>
-      </c>
-      <c r="F19" s="6">
-        <v>96.39</v>
-      </c>
-      <c r="G19" s="6">
-        <v>72.87</v>
-      </c>
-      <c r="H19" s="6">
-        <v>39.950000000000003</v>
-      </c>
-      <c r="I19" s="5">
-        <v>55.85</v>
+      <c r="A19" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="B19" s="16">
+        <v>88.35</v>
+      </c>
+      <c r="C19" s="16">
+        <v>71.25</v>
+      </c>
+      <c r="D19" s="17">
+        <v>95.67</v>
+      </c>
+      <c r="E19" s="16">
+        <v>65.78</v>
+      </c>
+      <c r="F19" s="16">
+        <v>96.3</v>
+      </c>
+      <c r="G19" s="16">
+        <v>72.5</v>
+      </c>
+      <c r="H19" s="16">
+        <v>37.590000000000003</v>
+      </c>
+      <c r="I19" s="16">
+        <v>56.72</v>
       </c>
     </row>
     <row r="20" spans="1:9">
       <c r="A20" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="B20" s="7">
+        <v>44</v>
+      </c>
+      <c r="B20" s="6">
         <v>89.11</v>
       </c>
-      <c r="C20" s="7">
+      <c r="C20" s="6">
         <v>72.12</v>
       </c>
-      <c r="D20" s="7">
+      <c r="D20" s="6">
         <v>95.83</v>
       </c>
-      <c r="E20" s="7">
+      <c r="E20" s="6">
         <v>66.13</v>
       </c>
-      <c r="F20" s="7">
+      <c r="F20" s="6">
         <v>96.49</v>
       </c>
-      <c r="G20" s="7">
+      <c r="G20" s="6">
         <v>73.63</v>
       </c>
-      <c r="H20" s="7">
+      <c r="H20" s="6">
         <v>40.22</v>
       </c>
-      <c r="I20" s="7">
+      <c r="I20" s="6">
         <v>54.17</v>
       </c>
     </row>
     <row r="21" spans="1:9">
       <c r="A21" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B21" s="7">
+        <v>45</v>
+      </c>
+      <c r="B21" s="6">
         <v>89.05</v>
       </c>
-      <c r="C21" s="7">
+      <c r="C21" s="6">
         <v>72.150000000000006</v>
       </c>
-      <c r="D21" s="7">
+      <c r="D21" s="6">
         <v>95.85</v>
       </c>
-      <c r="E21" s="7">
+      <c r="E21" s="6">
         <v>66.36</v>
       </c>
-      <c r="F21" s="7">
+      <c r="F21" s="6">
         <v>96.49</v>
       </c>
-      <c r="G21" s="7">
+      <c r="G21" s="6">
         <v>73.67</v>
       </c>
-      <c r="H21" s="7">
+      <c r="H21" s="6">
         <v>39.200000000000003</v>
       </c>
-      <c r="I21" s="7">
+      <c r="I21" s="6">
         <v>56.09</v>
       </c>
     </row>
     <row r="22" spans="1:9">
       <c r="A22" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="B22" s="9">
+        <v>46</v>
+      </c>
+      <c r="B22" s="8">
         <v>89.3</v>
       </c>
-      <c r="C22" s="7">
+      <c r="C22" s="6">
         <v>72.290000000000006</v>
       </c>
-      <c r="D22" s="9">
+      <c r="D22" s="8">
         <v>95.87</v>
       </c>
-      <c r="E22" s="7">
+      <c r="E22" s="6">
         <v>66.33</v>
       </c>
-      <c r="F22" s="9">
+      <c r="F22" s="8">
         <v>96.55</v>
       </c>
-      <c r="G22" s="9">
+      <c r="G22" s="8">
         <v>73.790000000000006</v>
       </c>
-      <c r="H22" s="7">
+      <c r="H22" s="6">
         <v>39.619999999999997</v>
       </c>
-      <c r="I22" s="7">
+      <c r="I22" s="6">
         <v>55.38</v>
       </c>
     </row>
     <row r="23" spans="1:9">
       <c r="A23" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="B23" s="7">
+        <v>47</v>
+      </c>
+      <c r="B23" s="6">
         <v>88.85</v>
       </c>
-      <c r="C23" s="7">
+      <c r="C23" s="6">
         <v>72.849999999999994</v>
       </c>
-      <c r="D23" s="7">
+      <c r="D23" s="6">
         <v>95.75</v>
       </c>
-      <c r="E23" s="7">
+      <c r="E23" s="6">
         <v>66.25</v>
       </c>
-      <c r="F23" s="7">
+      <c r="F23" s="6">
         <v>96.42</v>
       </c>
-      <c r="G23" s="7">
+      <c r="G23" s="6">
         <v>73.12</v>
       </c>
-      <c r="H23" s="9">
+      <c r="H23" s="8">
         <v>41.26</v>
       </c>
-      <c r="I23" s="7">
+      <c r="I23" s="6">
         <v>54.21</v>
       </c>
     </row>
     <row r="24" spans="1:9">
       <c r="A24" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="B24" s="7">
+        <v>48</v>
+      </c>
+      <c r="B24" s="6">
         <v>89.04</v>
       </c>
-      <c r="C24" s="9">
+      <c r="C24" s="8">
         <v>73.13</v>
       </c>
-      <c r="D24" s="7">
+      <c r="D24" s="6">
         <v>95.75</v>
       </c>
-      <c r="E24" s="9">
+      <c r="E24" s="8">
         <v>66.52</v>
       </c>
-      <c r="F24" s="7">
+      <c r="F24" s="6">
         <v>96.41</v>
       </c>
-      <c r="G24" s="7">
+      <c r="G24" s="6">
         <v>73.489999999999995</v>
       </c>
-      <c r="H24" s="7">
+      <c r="H24" s="6">
         <v>40.1</v>
       </c>
-      <c r="I24" s="7">
+      <c r="I24" s="6">
         <v>56.06</v>
       </c>
     </row>
     <row r="25" spans="1:9">
       <c r="A25" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="B25" s="7">
+        <v>49</v>
+      </c>
+      <c r="B25" s="6">
         <v>89.15</v>
       </c>
-      <c r="C25" s="7">
+      <c r="C25" s="6">
         <v>72.3</v>
       </c>
-      <c r="D25" s="7">
+      <c r="D25" s="6">
         <v>95.82</v>
       </c>
-      <c r="E25" s="7">
+      <c r="E25" s="6">
         <v>66.5</v>
       </c>
-      <c r="F25" s="7">
+      <c r="F25" s="6">
         <v>96.49</v>
       </c>
-      <c r="G25" s="7">
+      <c r="G25" s="6">
         <v>73.63</v>
       </c>
-      <c r="H25" s="7">
+      <c r="H25" s="6">
         <v>39.07</v>
       </c>
-      <c r="I25" s="9">
+      <c r="I25" s="8">
         <v>56.83</v>
       </c>
     </row>
     <row r="26" spans="1:9">
       <c r="A26" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B26" s="2">
         <v>87.36</v>
@@ -1890,12 +1903,12 @@
     </row>
     <row r="27" spans="1:9">
       <c r="A27" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B27" s="2">
         <v>87.68</v>
       </c>
-      <c r="C27" s="12">
+      <c r="C27" s="11">
         <v>71.77</v>
       </c>
       <c r="D27" s="2">
@@ -1919,7 +1932,7 @@
     </row>
     <row r="28" spans="1:9">
       <c r="A28" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B28" s="2">
         <v>86.59</v>
@@ -1948,7 +1961,7 @@
     </row>
     <row r="29" spans="1:9">
       <c r="A29" s="2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B29" s="2">
         <v>87.71</v>
@@ -1977,36 +1990,36 @@
     </row>
     <row r="30" spans="1:9">
       <c r="A30" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="B30" s="12">
+        <v>69</v>
+      </c>
+      <c r="B30" s="11">
         <v>88.79</v>
       </c>
       <c r="C30" s="2">
         <v>71.22</v>
       </c>
-      <c r="D30" s="12">
+      <c r="D30" s="11">
         <v>95.8</v>
       </c>
-      <c r="E30" s="12">
+      <c r="E30" s="11">
         <v>65.790000000000006</v>
       </c>
-      <c r="F30" s="12">
+      <c r="F30" s="11">
         <v>96.44</v>
       </c>
-      <c r="G30" s="12">
+      <c r="G30" s="11">
         <v>73.319999999999993</v>
       </c>
       <c r="H30" s="2">
         <v>39.26</v>
       </c>
-      <c r="I30" s="12">
+      <c r="I30" s="11">
         <v>54.12</v>
       </c>
     </row>
     <row r="31" spans="1:9">
       <c r="A31" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B31" s="2">
         <v>88.45</v>
@@ -2026,7 +2039,7 @@
       <c r="G31" s="2">
         <v>72.89</v>
       </c>
-      <c r="H31" s="12">
+      <c r="H31" s="11">
         <v>40.200000000000003</v>
       </c>
       <c r="I31" s="2">
@@ -2035,7 +2048,7 @@
     </row>
     <row r="32" spans="1:9">
       <c r="A32" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B32" s="3">
         <v>89.95</v>
@@ -2064,7 +2077,7 @@
     </row>
     <row r="33" spans="1:18">
       <c r="A33" s="3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B33" s="3">
         <v>90.11</v>
@@ -2084,7 +2097,7 @@
       <c r="G33" s="3">
         <v>74.08</v>
       </c>
-      <c r="H33" s="13">
+      <c r="H33" s="12">
         <v>42.35</v>
       </c>
       <c r="I33" s="3">
@@ -2093,7 +2106,7 @@
     </row>
     <row r="34" spans="1:18">
       <c r="A34" s="3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B34" s="3">
         <v>89.75</v>
@@ -2122,12 +2135,12 @@
     </row>
     <row r="35" spans="1:18">
       <c r="A35" s="3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B35" s="3">
         <v>89.93</v>
       </c>
-      <c r="C35" s="13">
+      <c r="C35" s="12">
         <v>74.41</v>
       </c>
       <c r="D35" s="3">
@@ -2151,7 +2164,7 @@
     </row>
     <row r="36" spans="1:18">
       <c r="A36" s="3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B36" s="3">
         <v>89.79</v>
@@ -2180,30 +2193,30 @@
     </row>
     <row r="37" spans="1:18">
       <c r="A37" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="B37" s="13">
+        <v>76</v>
+      </c>
+      <c r="B37" s="12">
         <v>90.12</v>
       </c>
       <c r="C37" s="3">
         <v>74.31</v>
       </c>
-      <c r="D37" s="13">
+      <c r="D37" s="12">
         <v>95.92</v>
       </c>
-      <c r="E37" s="13">
+      <c r="E37" s="12">
         <v>67.430000000000007</v>
       </c>
-      <c r="F37" s="13">
+      <c r="F37" s="12">
         <v>96.54</v>
       </c>
-      <c r="G37" s="13">
+      <c r="G37" s="12">
         <v>74.12</v>
       </c>
       <c r="H37" s="3">
         <v>41.82</v>
       </c>
-      <c r="I37" s="13">
+      <c r="I37" s="12">
         <v>57.25</v>
       </c>
     </row>
@@ -2261,22 +2274,22 @@
         <v>18</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>50</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>34</v>
@@ -2305,7 +2318,7 @@
         <v>41.28</v>
       </c>
       <c r="H2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -2331,7 +2344,7 @@
         <v>39.97</v>
       </c>
       <c r="H3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -2357,7 +2370,7 @@
         <v>60.83</v>
       </c>
       <c r="H4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -2383,7 +2396,7 @@
         <v>41.32</v>
       </c>
       <c r="H5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -2409,7 +2422,7 @@
         <v>68.87</v>
       </c>
       <c r="H6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -2435,7 +2448,7 @@
         <v>56.68</v>
       </c>
       <c r="H7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -2461,7 +2474,7 @@
         <v>46.65</v>
       </c>
       <c r="H8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -2487,7 +2500,7 @@
         <v>51.9</v>
       </c>
       <c r="H9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -2513,7 +2526,7 @@
         <v>45.75</v>
       </c>
       <c r="H10" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -2539,7 +2552,7 @@
         <v>58.28</v>
       </c>
       <c r="H11" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -2565,7 +2578,7 @@
         <v>43.25</v>
       </c>
       <c r="H12" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -2591,7 +2604,7 @@
         <v>62.24</v>
       </c>
       <c r="H13" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -2617,7 +2630,7 @@
         <v>51.87</v>
       </c>
       <c r="H14" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -2643,7 +2656,7 @@
         <v>41.34</v>
       </c>
       <c r="H15" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -2669,7 +2682,7 @@
         <v>50.73</v>
       </c>
       <c r="H16" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -2717,7 +2730,7 @@
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B2">
         <v>87.36</v>
@@ -2746,7 +2759,7 @@
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B3">
         <v>87.68</v>
@@ -2775,7 +2788,7 @@
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B4">
         <v>86.59</v>
@@ -2804,7 +2817,7 @@
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B5">
         <v>87.71</v>
@@ -2833,7 +2846,7 @@
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B6" s="1">
         <v>88.79</v>
@@ -2862,7 +2875,7 @@
     </row>
     <row r="7" spans="1:9">
       <c r="A7" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B7">
         <v>88.45</v>
@@ -2916,22 +2929,22 @@
         <v>18</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>70</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>72</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>34</v>
@@ -2941,390 +2954,390 @@
       <c r="A2" t="s">
         <v>19</v>
       </c>
-      <c r="B2" s="10">
+      <c r="B2" s="9">
         <v>41.76</v>
       </c>
-      <c r="C2" s="10">
+      <c r="C2" s="9">
         <v>39.4</v>
       </c>
-      <c r="D2" s="10">
+      <c r="D2" s="9">
         <v>38.72</v>
       </c>
-      <c r="E2" s="10">
+      <c r="E2" s="9">
         <v>42.78</v>
       </c>
-      <c r="F2" s="10">
+      <c r="F2" s="9">
         <v>41.75</v>
       </c>
-      <c r="G2" s="11">
+      <c r="G2" s="10">
         <v>45.26</v>
       </c>
       <c r="H2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" t="s">
         <v>20</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="9">
         <v>38.520000000000003</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="9">
         <v>39.200000000000003</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="9">
         <v>38.81</v>
       </c>
-      <c r="E3" s="11">
+      <c r="E3" s="10">
         <v>39.76</v>
       </c>
-      <c r="F3" s="10">
+      <c r="F3" s="9">
         <v>39.630000000000003</v>
       </c>
-      <c r="G3" s="10">
+      <c r="G3" s="9">
         <v>38.99</v>
       </c>
       <c r="H3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="9">
         <v>58.79</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="9">
         <v>61.49</v>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="9">
         <v>59.38</v>
       </c>
-      <c r="E4" s="11">
+      <c r="E4" s="10">
         <v>61.71</v>
       </c>
-      <c r="F4" s="10">
+      <c r="F4" s="9">
         <v>60.14</v>
       </c>
-      <c r="G4" s="10">
+      <c r="G4" s="9">
         <v>57.16</v>
       </c>
       <c r="H4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="10">
+      <c r="B5" s="9">
         <v>38.840000000000003</v>
       </c>
-      <c r="C5" s="10">
+      <c r="C5" s="9">
         <v>39.770000000000003</v>
       </c>
-      <c r="D5" s="10">
+      <c r="D5" s="9">
         <v>39.29</v>
       </c>
-      <c r="E5" s="10">
+      <c r="E5" s="9">
         <v>40.01</v>
       </c>
-      <c r="F5" s="11">
+      <c r="F5" s="10">
         <v>40.590000000000003</v>
       </c>
-      <c r="G5" s="10">
+      <c r="G5" s="9">
         <v>40.43</v>
       </c>
       <c r="H5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
         <v>23</v>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="9">
         <v>61.98</v>
       </c>
-      <c r="C6" s="11">
+      <c r="C6" s="10">
         <v>65.260000000000005</v>
       </c>
-      <c r="D6" s="10">
+      <c r="D6" s="9">
         <v>61.44</v>
       </c>
-      <c r="E6" s="10">
+      <c r="E6" s="9">
         <v>63.7</v>
       </c>
-      <c r="F6" s="10">
+      <c r="F6" s="9">
         <v>63.9</v>
       </c>
-      <c r="G6" s="10">
+      <c r="G6" s="9">
         <v>63.15</v>
       </c>
       <c r="H6" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" t="s">
         <v>24</v>
       </c>
-      <c r="B7" s="10">
+      <c r="B7" s="9">
         <v>40.950000000000003</v>
       </c>
-      <c r="C7" s="11">
+      <c r="C7" s="10">
         <v>53.97</v>
       </c>
-      <c r="D7" s="10">
+      <c r="D7" s="9">
         <v>49.33</v>
       </c>
-      <c r="E7" s="10">
+      <c r="E7" s="9">
         <v>45.88</v>
       </c>
-      <c r="F7" s="10">
+      <c r="F7" s="9">
         <v>48</v>
       </c>
-      <c r="G7" s="10">
+      <c r="G7" s="9">
         <v>48.95</v>
       </c>
       <c r="H7" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" t="s">
         <v>25</v>
       </c>
-      <c r="B8" s="10">
+      <c r="B8" s="9">
         <v>43.8</v>
       </c>
-      <c r="C8" s="10">
+      <c r="C8" s="9">
         <v>44.73</v>
       </c>
-      <c r="D8" s="10">
+      <c r="D8" s="9">
         <v>44.86</v>
       </c>
-      <c r="E8" s="10">
+      <c r="E8" s="9">
         <v>43.62</v>
       </c>
-      <c r="F8" s="10">
+      <c r="F8" s="9">
         <v>44.93</v>
       </c>
-      <c r="G8" s="11">
+      <c r="G8" s="10">
         <v>45.37</v>
       </c>
       <c r="H8" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="9" spans="1:8">
       <c r="A9" t="s">
         <v>26</v>
       </c>
-      <c r="B9" s="10">
+      <c r="B9" s="9">
         <v>49.41</v>
       </c>
-      <c r="C9" s="10">
+      <c r="C9" s="9">
         <v>50.16</v>
       </c>
-      <c r="D9" s="10">
+      <c r="D9" s="9">
         <v>47.49</v>
       </c>
-      <c r="E9" s="10">
+      <c r="E9" s="9">
         <v>50.48</v>
       </c>
-      <c r="F9" s="11">
+      <c r="F9" s="10">
         <v>50.67</v>
       </c>
-      <c r="G9" s="10">
+      <c r="G9" s="9">
         <v>49.74</v>
       </c>
       <c r="H9" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="10" spans="1:8">
       <c r="A10" t="s">
         <v>27</v>
       </c>
-      <c r="B10" s="11">
+      <c r="B10" s="10">
         <v>45.46</v>
       </c>
-      <c r="C10" s="10">
+      <c r="C10" s="9">
         <v>42.93</v>
       </c>
-      <c r="D10" s="10">
+      <c r="D10" s="9">
         <v>42.09</v>
       </c>
-      <c r="E10" s="10">
+      <c r="E10" s="9">
         <v>40.119999999999997</v>
       </c>
-      <c r="F10" s="10">
+      <c r="F10" s="9">
         <v>40.11</v>
       </c>
-      <c r="G10" s="10">
+      <c r="G10" s="9">
         <v>39.369999999999997</v>
       </c>
       <c r="H10" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" t="s">
         <v>28</v>
       </c>
-      <c r="B11" s="10">
+      <c r="B11" s="9">
         <v>55.86</v>
       </c>
-      <c r="C11" s="10">
+      <c r="C11" s="9">
         <v>56.15</v>
       </c>
-      <c r="D11" s="10">
+      <c r="D11" s="9">
         <v>54.39</v>
       </c>
-      <c r="E11" s="10">
+      <c r="E11" s="9">
         <v>57.85</v>
       </c>
-      <c r="F11" s="11">
+      <c r="F11" s="10">
         <v>58.71</v>
       </c>
-      <c r="G11" s="10">
+      <c r="G11" s="9">
         <v>57.17</v>
       </c>
       <c r="H11" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="12" spans="1:8">
       <c r="A12" t="s">
         <v>29</v>
       </c>
-      <c r="B12" s="10">
+      <c r="B12" s="9">
         <v>42.33</v>
       </c>
-      <c r="C12" s="10">
+      <c r="C12" s="9">
         <v>42.15</v>
       </c>
-      <c r="D12" s="10">
+      <c r="D12" s="9">
         <v>41.46</v>
       </c>
-      <c r="E12" s="10">
+      <c r="E12" s="9">
         <v>42.35</v>
       </c>
-      <c r="F12" s="11">
+      <c r="F12" s="10">
         <v>43.22</v>
       </c>
-      <c r="G12" s="10">
+      <c r="G12" s="9">
         <v>43.07</v>
       </c>
       <c r="H12" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="13" spans="1:8">
       <c r="A13" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="10">
+      <c r="B13" s="9">
         <v>53.77</v>
       </c>
-      <c r="C13" s="10">
+      <c r="C13" s="9">
         <v>56.58</v>
       </c>
-      <c r="D13" s="10">
+      <c r="D13" s="9">
         <v>52.53</v>
       </c>
-      <c r="E13" s="10">
+      <c r="E13" s="9">
         <v>53.92</v>
       </c>
-      <c r="F13" s="11">
+      <c r="F13" s="10">
         <v>60.73</v>
       </c>
-      <c r="G13" s="10">
+      <c r="G13" s="9">
         <v>57.28</v>
       </c>
       <c r="H13" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="14" spans="1:8">
       <c r="A14" t="s">
         <v>31</v>
       </c>
-      <c r="B14" s="10">
+      <c r="B14" s="9">
         <v>46.62</v>
       </c>
-      <c r="C14" s="10">
+      <c r="C14" s="9">
         <v>46.68</v>
       </c>
-      <c r="D14" s="10">
+      <c r="D14" s="9">
         <v>48.56</v>
       </c>
-      <c r="E14" s="11">
+      <c r="E14" s="10">
         <v>52.25</v>
       </c>
-      <c r="F14" s="10">
+      <c r="F14" s="9">
         <v>49.2</v>
       </c>
-      <c r="G14" s="10">
+      <c r="G14" s="9">
         <v>49.14</v>
       </c>
       <c r="H14" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="15" spans="1:8">
       <c r="A15" t="s">
         <v>32</v>
       </c>
-      <c r="B15" s="10">
+      <c r="B15" s="9">
         <v>36.96</v>
       </c>
-      <c r="C15" s="10">
+      <c r="C15" s="9">
         <v>38.15</v>
       </c>
-      <c r="D15" s="10">
+      <c r="D15" s="9">
         <v>37.54</v>
       </c>
-      <c r="E15" s="10">
+      <c r="E15" s="9">
         <v>40.39</v>
       </c>
-      <c r="F15" s="11">
+      <c r="F15" s="10">
         <v>45.54</v>
       </c>
-      <c r="G15" s="10">
+      <c r="G15" s="9">
         <v>40.81</v>
       </c>
       <c r="H15" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="16" spans="1:8">
       <c r="A16" t="s">
         <v>33</v>
       </c>
-      <c r="B16" s="10">
+      <c r="B16" s="9">
         <v>46.79</v>
       </c>
-      <c r="C16" s="10">
+      <c r="C16" s="9">
         <v>48.33</v>
       </c>
-      <c r="D16" s="10">
+      <c r="D16" s="9">
         <v>46.85</v>
       </c>
-      <c r="E16" s="10">
+      <c r="E16" s="9">
         <v>48.2</v>
       </c>
-      <c r="F16" s="11">
+      <c r="F16" s="10">
         <v>49.08</v>
       </c>
-      <c r="G16" s="10">
+      <c r="G16" s="9">
         <v>48.28</v>
       </c>
       <c r="H16" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -3372,7 +3385,7 @@
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B2">
         <v>89.95</v>
@@ -3401,7 +3414,7 @@
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B3">
         <v>90.11</v>
@@ -3430,7 +3443,7 @@
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B4">
         <v>89.75</v>
@@ -3459,7 +3472,7 @@
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B5">
         <v>89.93</v>
@@ -3488,7 +3501,7 @@
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B6">
         <v>89.79</v>
@@ -3517,7 +3530,7 @@
     </row>
     <row r="7" spans="1:9">
       <c r="A7" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B7" s="1">
         <v>90.12</v>
@@ -3570,22 +3583,22 @@
         <v>18</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>89</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>91</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>34</v>
@@ -3614,7 +3627,7 @@
         <v>53.89</v>
       </c>
       <c r="H2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -3640,7 +3653,7 @@
         <v>39.270000000000003</v>
       </c>
       <c r="H3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -3666,7 +3679,7 @@
         <v>61.58</v>
       </c>
       <c r="H4" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -3692,7 +3705,7 @@
         <v>41.27</v>
       </c>
       <c r="H5" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -3718,7 +3731,7 @@
         <v>63.99</v>
       </c>
       <c r="H6" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -3744,7 +3757,7 @@
         <v>57.8</v>
       </c>
       <c r="H7" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -3770,7 +3783,7 @@
         <v>46.65</v>
       </c>
       <c r="H8" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -3796,7 +3809,7 @@
         <v>54.56</v>
       </c>
       <c r="H9" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -3822,7 +3835,7 @@
         <v>44.65</v>
       </c>
       <c r="H10" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -3848,7 +3861,7 @@
         <v>57.92</v>
       </c>
       <c r="H11" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -3874,7 +3887,7 @@
         <v>43.35</v>
       </c>
       <c r="H12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -3900,7 +3913,7 @@
         <v>67.760000000000005</v>
       </c>
       <c r="H13" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -3926,7 +3939,7 @@
         <v>52.28</v>
       </c>
       <c r="H14" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -3952,7 +3965,7 @@
         <v>40.49</v>
       </c>
       <c r="H15" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -3978,7 +3991,7 @@
         <v>51.82</v>
       </c>
       <c r="H16" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>
@@ -4035,113 +4048,113 @@
       <c r="A1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="D1" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="E1" s="12" t="s">
+      <c r="D1" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="E1" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="G1" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="H1" s="13" t="s">
+      <c r="H1" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="I1" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="J1" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="K1" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="I1" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="J1" s="13" t="s">
+      <c r="L1" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="K1" s="13" t="s">
+      <c r="M1" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="L1" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="M1" s="13" t="s">
-        <v>64</v>
-      </c>
-      <c r="N1" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="O1" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="P1" s="12" t="s">
+      <c r="N1" s="17" t="s">
+        <v>94</v>
+      </c>
+      <c r="O1" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="P1" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="Q1" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="R1" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="S1" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="T1" s="13" t="s">
+      <c r="Q1" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="R1" s="17" t="s">
+        <v>91</v>
+      </c>
+      <c r="S1" s="17" t="s">
+        <v>93</v>
+      </c>
+      <c r="T1" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="U1" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="U1" s="13" t="s">
+      <c r="V1" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="V1" s="13" t="s">
+      <c r="W1" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="W1" s="13" t="s">
+      <c r="X1" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="X1" s="13" t="s">
+      <c r="Y1" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="Y1" s="13" t="s">
-        <v>50</v>
-      </c>
-      <c r="Z1" s="14" t="s">
+      <c r="Z1" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="AA1" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="AB1" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="AA1" s="14" t="s">
+      <c r="AC1" s="13" t="s">
         <v>68</v>
       </c>
-      <c r="AB1" s="14" t="s">
+      <c r="AD1" s="13" t="s">
         <v>69</v>
       </c>
-      <c r="AC1" s="14" t="s">
+      <c r="AE1" s="13" t="s">
         <v>70</v>
       </c>
-      <c r="AD1" s="14" t="s">
-        <v>71</v>
-      </c>
-      <c r="AE1" s="14" t="s">
+      <c r="AF1" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="AG1" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="AF1" s="13" t="s">
+      <c r="AH1" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="AI1" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="AJ1" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="AK1" s="12" t="s">
         <v>89</v>
-      </c>
-      <c r="AG1" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="AH1" s="13" t="s">
-        <v>75</v>
-      </c>
-      <c r="AI1" s="13" t="s">
-        <v>76</v>
-      </c>
-      <c r="AJ1" s="13" t="s">
-        <v>90</v>
-      </c>
-      <c r="AK1" s="13" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="2" spans="1:37">
@@ -4163,13 +4176,13 @@
       <c r="F2" s="2">
         <v>54.94</v>
       </c>
-      <c r="G2" s="12">
+      <c r="G2" s="11">
         <v>64.069999999999993</v>
       </c>
       <c r="H2" s="3">
         <v>52.77</v>
       </c>
-      <c r="I2" s="13">
+      <c r="I2" s="12">
         <v>54.63</v>
       </c>
       <c r="J2" s="3">
@@ -4184,28 +4197,28 @@
       <c r="M2" s="3">
         <v>48.69</v>
       </c>
-      <c r="N2" s="2">
+      <c r="N2" s="17">
         <v>56.81</v>
       </c>
-      <c r="O2" s="2">
+      <c r="O2" s="16">
         <v>48.12</v>
       </c>
-      <c r="P2" s="12">
+      <c r="P2" s="16">
         <v>59.15</v>
       </c>
-      <c r="Q2" s="2">
-        <v>45.78</v>
-      </c>
-      <c r="R2" s="2">
-        <v>48</v>
-      </c>
-      <c r="S2" s="2">
-        <v>52.73</v>
+      <c r="Q2" s="16">
+        <v>47.81</v>
+      </c>
+      <c r="R2" s="16">
+        <v>49.1</v>
+      </c>
+      <c r="S2" s="16">
+        <v>47.18</v>
       </c>
       <c r="T2" s="3">
         <v>48.07</v>
       </c>
-      <c r="U2" s="13">
+      <c r="U2" s="12">
         <v>48.11</v>
       </c>
       <c r="V2" s="3">
@@ -4220,22 +4233,22 @@
       <c r="Y2" s="3">
         <v>41.28</v>
       </c>
-      <c r="Z2" s="15">
+      <c r="Z2" s="14">
         <v>41.76</v>
       </c>
-      <c r="AA2" s="15">
+      <c r="AA2" s="14">
         <v>39.4</v>
       </c>
-      <c r="AB2" s="15">
+      <c r="AB2" s="14">
         <v>38.72</v>
       </c>
-      <c r="AC2" s="15">
+      <c r="AC2" s="14">
         <v>42.78</v>
       </c>
-      <c r="AD2" s="15">
+      <c r="AD2" s="14">
         <v>41.75</v>
       </c>
-      <c r="AE2" s="16">
+      <c r="AE2" s="15">
         <v>45.26</v>
       </c>
       <c r="AF2" s="3">
@@ -4247,7 +4260,7 @@
       <c r="AH2" s="3">
         <v>49.24</v>
       </c>
-      <c r="AI2" s="13">
+      <c r="AI2" s="12">
         <v>62.58</v>
       </c>
       <c r="AJ2" s="3">
@@ -4261,7 +4274,7 @@
       <c r="A3" t="s">
         <v>20</v>
       </c>
-      <c r="B3" s="12">
+      <c r="B3" s="11">
         <v>39.619999999999997</v>
       </c>
       <c r="C3" s="2">
@@ -4291,29 +4304,29 @@
       <c r="K3" s="3">
         <v>40.76</v>
       </c>
-      <c r="L3" s="13">
+      <c r="L3" s="12">
         <v>41.3</v>
       </c>
       <c r="M3" s="3">
         <v>39.97</v>
       </c>
-      <c r="N3" s="2">
+      <c r="N3" s="16">
         <v>39.61</v>
       </c>
-      <c r="O3" s="2">
+      <c r="O3" s="16">
         <v>39</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="16">
         <v>39.08</v>
       </c>
-      <c r="Q3" s="12">
-        <v>39.659999999999997</v>
-      </c>
-      <c r="R3" s="2">
-        <v>38.99</v>
-      </c>
-      <c r="S3" s="2">
-        <v>39.25</v>
+      <c r="Q3" s="16">
+        <v>38.96</v>
+      </c>
+      <c r="R3" s="17">
+        <v>39.82</v>
+      </c>
+      <c r="S3" s="16">
+        <v>39.32</v>
       </c>
       <c r="T3" s="3">
         <v>40.08</v>
@@ -4324,7 +4337,7 @@
       <c r="V3" s="3">
         <v>41.53</v>
       </c>
-      <c r="W3" s="13">
+      <c r="W3" s="12">
         <v>47.79</v>
       </c>
       <c r="X3" s="3">
@@ -4333,28 +4346,28 @@
       <c r="Y3" s="3">
         <v>39.97</v>
       </c>
-      <c r="Z3" s="15">
+      <c r="Z3" s="14">
         <v>38.520000000000003</v>
       </c>
-      <c r="AA3" s="15">
+      <c r="AA3" s="14">
         <v>39.200000000000003</v>
       </c>
-      <c r="AB3" s="15">
+      <c r="AB3" s="14">
         <v>38.81</v>
       </c>
-      <c r="AC3" s="16">
+      <c r="AC3" s="15">
         <v>39.76</v>
       </c>
-      <c r="AD3" s="15">
+      <c r="AD3" s="14">
         <v>39.630000000000003</v>
       </c>
-      <c r="AE3" s="15">
+      <c r="AE3" s="14">
         <v>38.99</v>
       </c>
       <c r="AF3" s="3">
         <v>39.44</v>
       </c>
-      <c r="AG3" s="13">
+      <c r="AG3" s="12">
         <v>39.94</v>
       </c>
       <c r="AH3" s="3">
@@ -4389,7 +4402,7 @@
       <c r="F4" s="2">
         <v>61.78</v>
       </c>
-      <c r="G4" s="12">
+      <c r="G4" s="11">
         <v>62.99</v>
       </c>
       <c r="H4" s="3">
@@ -4401,7 +4414,7 @@
       <c r="J4" s="3">
         <v>60.6</v>
       </c>
-      <c r="K4" s="13">
+      <c r="K4" s="12">
         <v>62.48</v>
       </c>
       <c r="L4" s="3">
@@ -4410,28 +4423,28 @@
       <c r="M4" s="3">
         <v>61.43</v>
       </c>
-      <c r="N4" s="2">
+      <c r="N4" s="16">
         <v>61.38</v>
       </c>
-      <c r="O4" s="2">
+      <c r="O4" s="16">
         <v>61.34</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="16">
         <v>60.81</v>
       </c>
-      <c r="Q4" s="2">
-        <v>60.95</v>
-      </c>
-      <c r="R4" s="2">
-        <v>61.06</v>
-      </c>
-      <c r="S4" s="2">
-        <v>60.93</v>
+      <c r="Q4" s="16">
+        <v>60.73</v>
+      </c>
+      <c r="R4" s="17">
+        <v>60.92</v>
+      </c>
+      <c r="S4" s="16">
+        <v>60.78</v>
       </c>
       <c r="T4" s="3">
         <v>59.83</v>
       </c>
-      <c r="U4" s="13">
+      <c r="U4" s="12">
         <v>61.8</v>
       </c>
       <c r="V4" s="3">
@@ -4446,22 +4459,22 @@
       <c r="Y4" s="3">
         <v>60.83</v>
       </c>
-      <c r="Z4" s="15">
+      <c r="Z4" s="14">
         <v>58.79</v>
       </c>
-      <c r="AA4" s="15">
+      <c r="AA4" s="14">
         <v>61.49</v>
       </c>
-      <c r="AB4" s="15">
+      <c r="AB4" s="14">
         <v>59.38</v>
       </c>
-      <c r="AC4" s="16">
+      <c r="AC4" s="15">
         <v>61.71</v>
       </c>
-      <c r="AD4" s="15">
+      <c r="AD4" s="14">
         <v>60.14</v>
       </c>
-      <c r="AE4" s="15">
+      <c r="AE4" s="14">
         <v>57.16</v>
       </c>
       <c r="AF4" s="3">
@@ -4502,10 +4515,10 @@
       <c r="F5" s="2">
         <v>41.43</v>
       </c>
-      <c r="G5" s="12">
+      <c r="G5" s="11">
         <v>41.74</v>
       </c>
-      <c r="H5" s="13">
+      <c r="H5" s="12">
         <v>42.1</v>
       </c>
       <c r="I5" s="3">
@@ -4523,23 +4536,23 @@
       <c r="M5" s="3">
         <v>41.87</v>
       </c>
-      <c r="N5" s="2">
+      <c r="N5" s="16">
         <v>40.17</v>
       </c>
-      <c r="O5" s="2">
+      <c r="O5" s="16">
         <v>40.71</v>
       </c>
-      <c r="P5" s="2">
+      <c r="P5" s="16">
         <v>40.770000000000003</v>
       </c>
-      <c r="Q5" s="12">
-        <v>41.41</v>
-      </c>
-      <c r="R5" s="2">
-        <v>40.86</v>
-      </c>
-      <c r="S5" s="2">
-        <v>40.659999999999997</v>
+      <c r="Q5" s="16">
+        <v>40.43</v>
+      </c>
+      <c r="R5" s="17">
+        <v>41.02</v>
+      </c>
+      <c r="S5" s="16">
+        <v>40.5</v>
       </c>
       <c r="T5" s="3">
         <v>41.37</v>
@@ -4547,7 +4560,7 @@
       <c r="U5" s="3">
         <v>41.35</v>
       </c>
-      <c r="V5" s="13">
+      <c r="V5" s="12">
         <v>41.55</v>
       </c>
       <c r="W5" s="3">
@@ -4559,28 +4572,28 @@
       <c r="Y5" s="3">
         <v>41.32</v>
       </c>
-      <c r="Z5" s="15">
+      <c r="Z5" s="14">
         <v>38.840000000000003</v>
       </c>
-      <c r="AA5" s="15">
+      <c r="AA5" s="14">
         <v>39.770000000000003</v>
       </c>
-      <c r="AB5" s="15">
+      <c r="AB5" s="14">
         <v>39.29</v>
       </c>
-      <c r="AC5" s="15">
+      <c r="AC5" s="14">
         <v>40.01</v>
       </c>
-      <c r="AD5" s="16">
+      <c r="AD5" s="15">
         <v>40.590000000000003</v>
       </c>
-      <c r="AE5" s="15">
+      <c r="AE5" s="14">
         <v>40.43</v>
       </c>
       <c r="AF5" s="3">
         <v>41.24</v>
       </c>
-      <c r="AG5" s="13">
+      <c r="AG5" s="12">
         <v>41.44</v>
       </c>
       <c r="AH5" s="3">
@@ -4615,7 +4628,7 @@
       <c r="F6" s="2">
         <v>62.54</v>
       </c>
-      <c r="G6" s="12">
+      <c r="G6" s="11">
         <v>63.01</v>
       </c>
       <c r="H6" s="3">
@@ -4630,29 +4643,29 @@
       <c r="K6" s="3">
         <v>64.39</v>
       </c>
-      <c r="L6" s="13">
+      <c r="L6" s="12">
         <v>65.14</v>
       </c>
       <c r="M6" s="3">
         <v>64.95</v>
       </c>
-      <c r="N6" s="2">
+      <c r="N6" s="16">
         <v>64.8</v>
       </c>
-      <c r="O6" s="2">
+      <c r="O6" s="16">
         <v>62.84</v>
       </c>
-      <c r="P6" s="12">
+      <c r="P6" s="16">
         <v>66.8</v>
       </c>
-      <c r="Q6" s="2">
-        <v>62.92</v>
-      </c>
-      <c r="R6" s="2">
-        <v>64.930000000000007</v>
-      </c>
-      <c r="S6" s="2">
-        <v>64.040000000000006</v>
+      <c r="Q6" s="17">
+        <v>67.78</v>
+      </c>
+      <c r="R6" s="16">
+        <v>65.900000000000006</v>
+      </c>
+      <c r="S6" s="16">
+        <v>65.28</v>
       </c>
       <c r="T6" s="3">
         <v>63.46</v>
@@ -4669,25 +4682,25 @@
       <c r="X6" s="3">
         <v>64.239999999999995</v>
       </c>
-      <c r="Y6" s="13">
+      <c r="Y6" s="12">
         <v>68.87</v>
       </c>
-      <c r="Z6" s="15">
+      <c r="Z6" s="14">
         <v>61.98</v>
       </c>
-      <c r="AA6" s="16">
+      <c r="AA6" s="15">
         <v>65.260000000000005</v>
       </c>
-      <c r="AB6" s="15">
+      <c r="AB6" s="14">
         <v>61.44</v>
       </c>
-      <c r="AC6" s="15">
+      <c r="AC6" s="14">
         <v>63.7</v>
       </c>
-      <c r="AD6" s="15">
+      <c r="AD6" s="14">
         <v>63.9</v>
       </c>
-      <c r="AE6" s="15">
+      <c r="AE6" s="14">
         <v>63.15</v>
       </c>
       <c r="AF6" s="3">
@@ -4699,7 +4712,7 @@
       <c r="AH6" s="3">
         <v>64.599999999999994</v>
       </c>
-      <c r="AI6" s="13">
+      <c r="AI6" s="12">
         <v>64.97</v>
       </c>
       <c r="AJ6" s="3">
@@ -4728,13 +4741,13 @@
       <c r="F7" s="2">
         <v>53.92</v>
       </c>
-      <c r="G7" s="12">
+      <c r="G7" s="11">
         <v>57.56</v>
       </c>
       <c r="H7" s="3">
         <v>57.72</v>
       </c>
-      <c r="I7" s="13">
+      <c r="I7" s="12">
         <v>59.02</v>
       </c>
       <c r="J7" s="3">
@@ -4749,23 +4762,23 @@
       <c r="M7" s="3">
         <v>56.4</v>
       </c>
-      <c r="N7" s="2">
+      <c r="N7" s="16">
         <v>45.66</v>
       </c>
-      <c r="O7" s="2">
+      <c r="O7" s="16">
         <v>50.67</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="16">
         <v>49.56</v>
       </c>
-      <c r="Q7" s="2">
-        <v>52.68</v>
-      </c>
-      <c r="R7" s="12">
-        <v>53.18</v>
-      </c>
-      <c r="S7" s="2">
-        <v>51.53</v>
+      <c r="Q7" s="16">
+        <v>49.4</v>
+      </c>
+      <c r="R7" s="16">
+        <v>53.09</v>
+      </c>
+      <c r="S7" s="17">
+        <v>53.27</v>
       </c>
       <c r="T7" s="3">
         <v>55.58</v>
@@ -4773,7 +4786,7 @@
       <c r="U7" s="3">
         <v>57.4</v>
       </c>
-      <c r="V7" s="13">
+      <c r="V7" s="12">
         <v>57.44</v>
       </c>
       <c r="W7" s="3">
@@ -4785,22 +4798,22 @@
       <c r="Y7" s="3">
         <v>56.68</v>
       </c>
-      <c r="Z7" s="15">
+      <c r="Z7" s="14">
         <v>40.950000000000003</v>
       </c>
-      <c r="AA7" s="16">
+      <c r="AA7" s="15">
         <v>53.97</v>
       </c>
-      <c r="AB7" s="15">
+      <c r="AB7" s="14">
         <v>49.33</v>
       </c>
-      <c r="AC7" s="15">
+      <c r="AC7" s="14">
         <v>45.88</v>
       </c>
-      <c r="AD7" s="15">
+      <c r="AD7" s="14">
         <v>48</v>
       </c>
-      <c r="AE7" s="15">
+      <c r="AE7" s="14">
         <v>48.95</v>
       </c>
       <c r="AF7" s="3">
@@ -4818,7 +4831,7 @@
       <c r="AJ7" s="3">
         <v>55.85</v>
       </c>
-      <c r="AK7" s="13">
+      <c r="AK7" s="12">
         <v>57.8</v>
       </c>
     </row>
@@ -4841,7 +4854,7 @@
       <c r="F8" s="2">
         <v>46.22</v>
       </c>
-      <c r="G8" s="12">
+      <c r="G8" s="11">
         <v>46.56</v>
       </c>
       <c r="H8" s="3">
@@ -4853,7 +4866,7 @@
       <c r="J8" s="3">
         <v>46.88</v>
       </c>
-      <c r="K8" s="13">
+      <c r="K8" s="12">
         <v>47.87</v>
       </c>
       <c r="L8" s="3">
@@ -4862,23 +4875,23 @@
       <c r="M8" s="3">
         <v>46.6</v>
       </c>
-      <c r="N8" s="2">
+      <c r="N8" s="16">
         <v>43.94</v>
       </c>
-      <c r="O8" s="2">
+      <c r="O8" s="16">
         <v>44.85</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="16">
         <v>43.63</v>
       </c>
-      <c r="Q8" s="2">
-        <v>44.59</v>
-      </c>
-      <c r="R8" s="2">
-        <v>45</v>
-      </c>
-      <c r="S8" s="12">
-        <v>45.02</v>
+      <c r="Q8" s="16">
+        <v>44.02</v>
+      </c>
+      <c r="R8" s="16">
+        <v>44.11</v>
+      </c>
+      <c r="S8" s="17">
+        <v>44.76</v>
       </c>
       <c r="T8" s="3">
         <v>46.74</v>
@@ -4886,7 +4899,7 @@
       <c r="U8" s="3">
         <v>45.98</v>
       </c>
-      <c r="V8" s="13">
+      <c r="V8" s="12">
         <v>46.77</v>
       </c>
       <c r="W8" s="3">
@@ -4898,22 +4911,22 @@
       <c r="Y8" s="3">
         <v>46.65</v>
       </c>
-      <c r="Z8" s="15">
+      <c r="Z8" s="14">
         <v>43.8</v>
       </c>
-      <c r="AA8" s="15">
+      <c r="AA8" s="14">
         <v>44.73</v>
       </c>
-      <c r="AB8" s="15">
+      <c r="AB8" s="14">
         <v>44.86</v>
       </c>
-      <c r="AC8" s="15">
+      <c r="AC8" s="14">
         <v>43.62</v>
       </c>
-      <c r="AD8" s="15">
+      <c r="AD8" s="14">
         <v>44.93</v>
       </c>
-      <c r="AE8" s="16">
+      <c r="AE8" s="15">
         <v>45.37</v>
       </c>
       <c r="AF8" s="3">
@@ -4922,7 +4935,7 @@
       <c r="AG8" s="3">
         <v>46.41</v>
       </c>
-      <c r="AH8" s="13">
+      <c r="AH8" s="12">
         <v>46.9</v>
       </c>
       <c r="AI8" s="3">
@@ -4951,7 +4964,7 @@
       <c r="E9" s="2">
         <v>52.03</v>
       </c>
-      <c r="F9" s="12">
+      <c r="F9" s="11">
         <v>53.81</v>
       </c>
       <c r="G9" s="2">
@@ -4966,7 +4979,7 @@
       <c r="J9" s="3">
         <v>51.9</v>
       </c>
-      <c r="K9" s="13">
+      <c r="K9" s="12">
         <v>52.51</v>
       </c>
       <c r="L9" s="3">
@@ -4975,23 +4988,23 @@
       <c r="M9" s="3">
         <v>51.69</v>
       </c>
-      <c r="N9" s="2">
+      <c r="N9" s="16">
         <v>48.91</v>
       </c>
-      <c r="O9" s="2">
+      <c r="O9" s="16">
         <v>47.94</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="16">
         <v>49.04</v>
       </c>
-      <c r="Q9" s="2">
-        <v>46.97</v>
-      </c>
-      <c r="R9" s="12">
-        <v>49.74</v>
-      </c>
-      <c r="S9" s="2">
-        <v>48.25</v>
+      <c r="Q9" s="16">
+        <v>48.18</v>
+      </c>
+      <c r="R9" s="17">
+        <v>49.32</v>
+      </c>
+      <c r="S9" s="16">
+        <v>48.52</v>
       </c>
       <c r="T9" s="3">
         <v>52.98</v>
@@ -5005,28 +5018,28 @@
       <c r="W9" s="3">
         <v>50.81</v>
       </c>
-      <c r="X9" s="13">
+      <c r="X9" s="12">
         <v>53.3</v>
       </c>
       <c r="Y9" s="3">
         <v>51.9</v>
       </c>
-      <c r="Z9" s="15">
+      <c r="Z9" s="14">
         <v>49.41</v>
       </c>
-      <c r="AA9" s="15">
+      <c r="AA9" s="14">
         <v>50.16</v>
       </c>
-      <c r="AB9" s="15">
+      <c r="AB9" s="14">
         <v>47.49</v>
       </c>
-      <c r="AC9" s="15">
+      <c r="AC9" s="14">
         <v>50.48</v>
       </c>
-      <c r="AD9" s="16">
+      <c r="AD9" s="15">
         <v>50.67</v>
       </c>
-      <c r="AE9" s="15">
+      <c r="AE9" s="14">
         <v>49.74</v>
       </c>
       <c r="AF9" s="3">
@@ -5044,7 +5057,7 @@
       <c r="AJ9" s="3">
         <v>49.79</v>
       </c>
-      <c r="AK9" s="13">
+      <c r="AK9" s="12">
         <v>54.56</v>
       </c>
     </row>
@@ -5067,7 +5080,7 @@
       <c r="F10" s="2">
         <v>42.57</v>
       </c>
-      <c r="G10" s="12">
+      <c r="G10" s="11">
         <v>45.56</v>
       </c>
       <c r="H10" s="3">
@@ -5082,29 +5095,29 @@
       <c r="K10" s="3">
         <v>45.19</v>
       </c>
-      <c r="L10" s="13">
+      <c r="L10" s="12">
         <v>49.29</v>
       </c>
       <c r="M10" s="3">
         <v>48.2</v>
       </c>
-      <c r="N10" s="2">
+      <c r="N10" s="16">
         <v>38.770000000000003</v>
       </c>
-      <c r="O10" s="2">
+      <c r="O10" s="16">
         <v>40.33</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="16">
         <v>38.08</v>
       </c>
-      <c r="Q10" s="12">
-        <v>40.83</v>
-      </c>
-      <c r="R10" s="2">
-        <v>38.659999999999997</v>
-      </c>
-      <c r="S10" s="2">
-        <v>40.130000000000003</v>
+      <c r="Q10" s="16">
+        <v>39.81</v>
+      </c>
+      <c r="R10" s="16">
+        <v>40.98</v>
+      </c>
+      <c r="S10" s="17">
+        <v>42.68</v>
       </c>
       <c r="T10" s="3">
         <v>43.16</v>
@@ -5121,25 +5134,25 @@
       <c r="X10" s="3">
         <v>42.4</v>
       </c>
-      <c r="Y10" s="13">
+      <c r="Y10" s="12">
         <v>45.75</v>
       </c>
-      <c r="Z10" s="16">
+      <c r="Z10" s="15">
         <v>45.46</v>
       </c>
-      <c r="AA10" s="15">
+      <c r="AA10" s="14">
         <v>42.93</v>
       </c>
-      <c r="AB10" s="15">
+      <c r="AB10" s="14">
         <v>42.09</v>
       </c>
-      <c r="AC10" s="15">
+      <c r="AC10" s="14">
         <v>40.119999999999997</v>
       </c>
-      <c r="AD10" s="15">
+      <c r="AD10" s="14">
         <v>40.11</v>
       </c>
-      <c r="AE10" s="15">
+      <c r="AE10" s="14">
         <v>39.369999999999997</v>
       </c>
       <c r="AF10" s="3">
@@ -5157,7 +5170,7 @@
       <c r="AJ10" s="3">
         <v>42.1</v>
       </c>
-      <c r="AK10" s="13">
+      <c r="AK10" s="12">
         <v>44.65</v>
       </c>
     </row>
@@ -5180,7 +5193,7 @@
       <c r="F11" s="2">
         <v>57.96</v>
       </c>
-      <c r="G11" s="12">
+      <c r="G11" s="11">
         <v>58.32</v>
       </c>
       <c r="H11" s="3">
@@ -5192,7 +5205,7 @@
       <c r="J11" s="3">
         <v>60.57</v>
       </c>
-      <c r="K11" s="13">
+      <c r="K11" s="12">
         <v>61.08</v>
       </c>
       <c r="L11" s="3">
@@ -5201,25 +5214,25 @@
       <c r="M11" s="3">
         <v>60.94</v>
       </c>
-      <c r="N11" s="2">
+      <c r="N11" s="16">
         <v>47.2</v>
       </c>
-      <c r="O11" s="2">
+      <c r="O11" s="16">
         <v>57.08</v>
       </c>
-      <c r="P11" s="12">
+      <c r="P11" s="16">
         <v>60.31</v>
       </c>
-      <c r="Q11" s="2">
-        <v>56.52</v>
-      </c>
-      <c r="R11" s="2">
-        <v>56.85</v>
-      </c>
-      <c r="S11" s="2">
-        <v>54.99</v>
-      </c>
-      <c r="T11" s="13">
+      <c r="Q11" s="16">
+        <v>51.04</v>
+      </c>
+      <c r="R11" s="17">
+        <v>59.25</v>
+      </c>
+      <c r="S11" s="16">
+        <v>58.88</v>
+      </c>
+      <c r="T11" s="12">
         <v>60.61</v>
       </c>
       <c r="U11" s="3">
@@ -5237,22 +5250,22 @@
       <c r="Y11" s="3">
         <v>58.28</v>
       </c>
-      <c r="Z11" s="15">
+      <c r="Z11" s="14">
         <v>55.86</v>
       </c>
-      <c r="AA11" s="15">
+      <c r="AA11" s="14">
         <v>56.15</v>
       </c>
-      <c r="AB11" s="15">
+      <c r="AB11" s="14">
         <v>54.39</v>
       </c>
-      <c r="AC11" s="15">
+      <c r="AC11" s="14">
         <v>57.85</v>
       </c>
-      <c r="AD11" s="16">
+      <c r="AD11" s="15">
         <v>58.71</v>
       </c>
-      <c r="AE11" s="15">
+      <c r="AE11" s="14">
         <v>57.17</v>
       </c>
       <c r="AF11" s="3">
@@ -5264,7 +5277,7 @@
       <c r="AH11" s="3">
         <v>57.48</v>
       </c>
-      <c r="AI11" s="13">
+      <c r="AI11" s="12">
         <v>59.18</v>
       </c>
       <c r="AJ11" s="3">
@@ -5293,10 +5306,10 @@
       <c r="F12" s="2">
         <v>43.4</v>
       </c>
-      <c r="G12" s="12">
+      <c r="G12" s="11">
         <v>43.59</v>
       </c>
-      <c r="H12" s="13">
+      <c r="H12" s="12">
         <v>45.87</v>
       </c>
       <c r="I12" s="3">
@@ -5314,25 +5327,25 @@
       <c r="M12" s="3">
         <v>44.14</v>
       </c>
-      <c r="N12" s="2">
+      <c r="N12" s="16">
         <v>42.98</v>
       </c>
-      <c r="O12" s="2">
+      <c r="O12" s="16">
         <v>42.94</v>
       </c>
-      <c r="P12" s="2">
+      <c r="P12" s="16">
         <v>42.75</v>
       </c>
-      <c r="Q12" s="2">
-        <v>42.91</v>
-      </c>
-      <c r="R12" s="12">
-        <v>43.32</v>
-      </c>
-      <c r="S12" s="2">
-        <v>43.06</v>
-      </c>
-      <c r="T12" s="13">
+      <c r="Q12" s="16">
+        <v>42.58</v>
+      </c>
+      <c r="R12" s="17">
+        <v>43.01</v>
+      </c>
+      <c r="S12" s="16">
+        <v>42.76</v>
+      </c>
+      <c r="T12" s="12">
         <v>43.36</v>
       </c>
       <c r="U12" s="3">
@@ -5350,22 +5363,22 @@
       <c r="Y12" s="3">
         <v>43.25</v>
       </c>
-      <c r="Z12" s="15">
+      <c r="Z12" s="14">
         <v>42.33</v>
       </c>
-      <c r="AA12" s="15">
+      <c r="AA12" s="14">
         <v>42.15</v>
       </c>
-      <c r="AB12" s="15">
+      <c r="AB12" s="14">
         <v>41.46</v>
       </c>
-      <c r="AC12" s="15">
+      <c r="AC12" s="14">
         <v>42.35</v>
       </c>
-      <c r="AD12" s="16">
+      <c r="AD12" s="15">
         <v>43.22</v>
       </c>
-      <c r="AE12" s="15">
+      <c r="AE12" s="14">
         <v>43.07</v>
       </c>
       <c r="AF12" s="3">
@@ -5383,7 +5396,7 @@
       <c r="AJ12" s="3">
         <v>43.03</v>
       </c>
-      <c r="AK12" s="13">
+      <c r="AK12" s="12">
         <v>43.35</v>
       </c>
     </row>
@@ -5403,7 +5416,7 @@
       <c r="E13" s="2">
         <v>56.94</v>
       </c>
-      <c r="F13" s="12">
+      <c r="F13" s="11">
         <v>66.069999999999993</v>
       </c>
       <c r="G13" s="2">
@@ -5424,26 +5437,26 @@
       <c r="L13" s="3">
         <v>62.1</v>
       </c>
-      <c r="M13" s="13">
+      <c r="M13" s="12">
         <v>64.66</v>
       </c>
-      <c r="N13" s="2">
+      <c r="N13" s="16">
         <v>62.23</v>
       </c>
-      <c r="O13" s="2">
+      <c r="O13" s="16">
         <v>63.36</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="16">
         <v>63.88</v>
       </c>
-      <c r="Q13" s="2">
-        <v>57.62</v>
-      </c>
-      <c r="R13" s="2">
-        <v>59.57</v>
-      </c>
-      <c r="S13" s="12">
-        <v>64.680000000000007</v>
+      <c r="Q13" s="16">
+        <v>67.08</v>
+      </c>
+      <c r="R13" s="17">
+        <v>68.52</v>
+      </c>
+      <c r="S13" s="16">
+        <v>63.84</v>
       </c>
       <c r="T13" s="3">
         <v>57.22</v>
@@ -5457,34 +5470,34 @@
       <c r="W13" s="3">
         <v>60.4</v>
       </c>
-      <c r="X13" s="13">
+      <c r="X13" s="12">
         <v>62.97</v>
       </c>
       <c r="Y13" s="3">
         <v>62.24</v>
       </c>
-      <c r="Z13" s="15">
+      <c r="Z13" s="14">
         <v>53.77</v>
       </c>
-      <c r="AA13" s="15">
+      <c r="AA13" s="14">
         <v>56.58</v>
       </c>
-      <c r="AB13" s="15">
+      <c r="AB13" s="14">
         <v>52.53</v>
       </c>
-      <c r="AC13" s="15">
+      <c r="AC13" s="14">
         <v>53.92</v>
       </c>
-      <c r="AD13" s="16">
+      <c r="AD13" s="15">
         <v>60.73</v>
       </c>
-      <c r="AE13" s="15">
+      <c r="AE13" s="14">
         <v>57.28</v>
       </c>
       <c r="AF13" s="3">
         <v>63.29</v>
       </c>
-      <c r="AG13" s="13">
+      <c r="AG13" s="12">
         <v>68.959999999999994</v>
       </c>
       <c r="AH13" s="3">
@@ -5516,7 +5529,7 @@
       <c r="E14" s="2">
         <v>39.51</v>
       </c>
-      <c r="F14" s="12">
+      <c r="F14" s="11">
         <v>51.55</v>
       </c>
       <c r="G14" s="2">
@@ -5534,29 +5547,29 @@
       <c r="K14" s="3">
         <v>53.04</v>
       </c>
-      <c r="L14" s="13">
+      <c r="L14" s="12">
         <v>54.87</v>
       </c>
       <c r="M14" s="3">
         <v>54.69</v>
       </c>
-      <c r="N14" s="2">
+      <c r="N14" s="16">
         <v>42.37</v>
       </c>
-      <c r="O14" s="2">
+      <c r="O14" s="16">
         <v>44.42</v>
       </c>
-      <c r="P14" s="12">
+      <c r="P14" s="16">
         <v>53.15</v>
       </c>
-      <c r="Q14" s="2">
-        <v>42.91</v>
-      </c>
-      <c r="R14" s="2">
-        <v>46.08</v>
-      </c>
-      <c r="S14" s="2">
-        <v>50.97</v>
+      <c r="Q14" s="16">
+        <v>39.619999999999997</v>
+      </c>
+      <c r="R14" s="16">
+        <v>44.42</v>
+      </c>
+      <c r="S14" s="16">
+        <v>41.62</v>
       </c>
       <c r="T14" s="3">
         <v>53.47</v>
@@ -5564,7 +5577,7 @@
       <c r="U14" s="3">
         <v>52.17</v>
       </c>
-      <c r="V14" s="13">
+      <c r="V14" s="12">
         <v>54.69</v>
       </c>
       <c r="W14" s="3">
@@ -5576,22 +5589,22 @@
       <c r="Y14" s="3">
         <v>51.87</v>
       </c>
-      <c r="Z14" s="15">
+      <c r="Z14" s="14">
         <v>46.62</v>
       </c>
-      <c r="AA14" s="15">
+      <c r="AA14" s="14">
         <v>46.68</v>
       </c>
-      <c r="AB14" s="15">
+      <c r="AB14" s="14">
         <v>48.56</v>
       </c>
-      <c r="AC14" s="16">
+      <c r="AC14" s="15">
         <v>52.25</v>
       </c>
-      <c r="AD14" s="15">
+      <c r="AD14" s="14">
         <v>49.2</v>
       </c>
-      <c r="AE14" s="15">
+      <c r="AE14" s="14">
         <v>49.14</v>
       </c>
       <c r="AF14" s="3">
@@ -5606,7 +5619,7 @@
       <c r="AI14" s="3">
         <v>51.66</v>
       </c>
-      <c r="AJ14" s="13">
+      <c r="AJ14" s="12">
         <v>54.75</v>
       </c>
       <c r="AK14" s="3">
@@ -5626,7 +5639,7 @@
       <c r="D15" s="2">
         <v>36.39</v>
       </c>
-      <c r="E15" s="12">
+      <c r="E15" s="11">
         <v>42.14</v>
       </c>
       <c r="F15" s="2">
@@ -5644,7 +5657,7 @@
       <c r="J15" s="3">
         <v>42.8</v>
       </c>
-      <c r="K15" s="13">
+      <c r="K15" s="12">
         <v>46.95</v>
       </c>
       <c r="L15" s="3">
@@ -5653,23 +5666,23 @@
       <c r="M15" s="3">
         <v>39.020000000000003</v>
       </c>
-      <c r="N15" s="12">
+      <c r="N15" s="16">
         <v>44.04</v>
       </c>
-      <c r="O15" s="2">
+      <c r="O15" s="16">
         <v>37.79</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="16">
         <v>36.979999999999997</v>
       </c>
-      <c r="Q15" s="2">
-        <v>39.5</v>
-      </c>
-      <c r="R15" s="2">
-        <v>38.51</v>
-      </c>
-      <c r="S15" s="2">
-        <v>37.78</v>
+      <c r="Q15" s="17">
+        <v>44.21</v>
+      </c>
+      <c r="R15" s="16">
+        <v>38.46</v>
+      </c>
+      <c r="S15" s="16">
+        <v>36.520000000000003</v>
       </c>
       <c r="T15" s="3">
         <v>38.08</v>
@@ -5683,28 +5696,28 @@
       <c r="W15" s="3">
         <v>40.85</v>
       </c>
-      <c r="X15" s="13">
+      <c r="X15" s="12">
         <v>42.36</v>
       </c>
       <c r="Y15" s="3">
         <v>41.34</v>
       </c>
-      <c r="Z15" s="15">
+      <c r="Z15" s="14">
         <v>36.96</v>
       </c>
-      <c r="AA15" s="15">
+      <c r="AA15" s="14">
         <v>38.15</v>
       </c>
-      <c r="AB15" s="15">
+      <c r="AB15" s="14">
         <v>37.54</v>
       </c>
-      <c r="AC15" s="15">
+      <c r="AC15" s="14">
         <v>40.39</v>
       </c>
-      <c r="AD15" s="16">
+      <c r="AD15" s="15">
         <v>45.54</v>
       </c>
-      <c r="AE15" s="15">
+      <c r="AE15" s="14">
         <v>40.81</v>
       </c>
       <c r="AF15" s="3">
@@ -5722,7 +5735,7 @@
       <c r="AJ15" s="3">
         <v>38.950000000000003</v>
       </c>
-      <c r="AK15" s="13">
+      <c r="AK15" s="12">
         <v>40.49</v>
       </c>
     </row>
@@ -5745,10 +5758,10 @@
       <c r="F16" s="2">
         <v>51.09</v>
       </c>
-      <c r="G16" s="12">
+      <c r="G16" s="11">
         <v>51.59</v>
       </c>
-      <c r="H16" s="13">
+      <c r="H16" s="12">
         <v>52.04</v>
       </c>
       <c r="I16" s="3">
@@ -5766,23 +5779,23 @@
       <c r="M16" s="3">
         <v>51.66</v>
       </c>
-      <c r="N16" s="2">
+      <c r="N16" s="16">
         <v>48.49</v>
       </c>
-      <c r="O16" s="2">
+      <c r="O16" s="16">
         <v>48.67</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="16">
         <v>50.29</v>
       </c>
-      <c r="Q16" s="2">
-        <v>48.23</v>
-      </c>
-      <c r="R16" s="2">
-        <v>48.91</v>
-      </c>
-      <c r="S16" s="12">
-        <v>49.57</v>
+      <c r="Q16" s="16">
+        <v>48.69</v>
+      </c>
+      <c r="R16" s="17">
+        <v>49.85</v>
+      </c>
+      <c r="S16" s="16">
+        <v>48.99</v>
       </c>
       <c r="T16" s="3">
         <v>50.29</v>
@@ -5796,28 +5809,28 @@
       <c r="W16" s="3">
         <v>50.52</v>
       </c>
-      <c r="X16" s="13">
+      <c r="X16" s="12">
         <v>51.11</v>
       </c>
       <c r="Y16" s="3">
         <v>50.73</v>
       </c>
-      <c r="Z16" s="15">
+      <c r="Z16" s="14">
         <v>46.79</v>
       </c>
-      <c r="AA16" s="15">
+      <c r="AA16" s="14">
         <v>48.33</v>
       </c>
-      <c r="AB16" s="15">
+      <c r="AB16" s="14">
         <v>46.85</v>
       </c>
-      <c r="AC16" s="15">
+      <c r="AC16" s="14">
         <v>48.2</v>
       </c>
-      <c r="AD16" s="16">
+      <c r="AD16" s="15">
         <v>49.08</v>
       </c>
-      <c r="AE16" s="15">
+      <c r="AE16" s="14">
         <v>48.28</v>
       </c>
       <c r="AF16" s="3">
@@ -5835,7 +5848,7 @@
       <c r="AJ16" s="3">
         <v>49.54</v>
       </c>
-      <c r="AK16" s="13">
+      <c r="AK16" s="12">
         <v>51.82</v>
       </c>
     </row>
@@ -6062,7 +6075,7 @@
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B4">
         <v>88.07</v>
@@ -6195,7 +6208,7 @@
     <col min="5" max="5" width="32" customWidth="1"/>
     <col min="6" max="6" width="31.1640625" customWidth="1"/>
     <col min="7" max="7" width="30.1640625" customWidth="1"/>
-    <col min="8" max="8" width="23.6640625" customWidth="1"/>
+    <col min="8" max="8" width="34.1640625" customWidth="1"/>
     <col min="9" max="9" width="41.1640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -6210,7 +6223,7 @@
         <v>10</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>15</v>
@@ -6220,6 +6233,9 @@
       </c>
       <c r="G1" s="1" t="s">
         <v>17</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -6244,12 +6260,15 @@
       <c r="G2" s="1">
         <v>64.069999999999993</v>
       </c>
+      <c r="H2" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
         <v>20</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B3" s="18">
         <v>39.619999999999997</v>
       </c>
       <c r="C3">
@@ -6261,11 +6280,14 @@
       <c r="E3">
         <v>39.479999999999997</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="1">
         <v>41.12</v>
       </c>
       <c r="G3">
         <v>39.54</v>
+      </c>
+      <c r="H3" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -6290,6 +6312,9 @@
       <c r="G4" s="1">
         <v>62.99</v>
       </c>
+      <c r="H4" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
@@ -6313,6 +6338,9 @@
       <c r="G5" s="1">
         <v>41.74</v>
       </c>
+      <c r="H5" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
@@ -6336,6 +6364,9 @@
       <c r="G6" s="1">
         <v>63.01</v>
       </c>
+      <c r="H6" t="s">
+        <v>17</v>
+      </c>
       <c r="I6" s="1"/>
     </row>
     <row r="7" spans="1:9">
@@ -6360,6 +6391,9 @@
       <c r="G7" s="1">
         <v>57.56</v>
       </c>
+      <c r="H7" t="s">
+        <v>17</v>
+      </c>
       <c r="I7" s="1"/>
     </row>
     <row r="8" spans="1:9">
@@ -6384,6 +6418,9 @@
       <c r="G8" s="1">
         <v>46.56</v>
       </c>
+      <c r="H8" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="9" spans="1:9">
       <c r="A9" t="s">
@@ -6407,6 +6444,9 @@
       <c r="G9">
         <v>51.49</v>
       </c>
+      <c r="H9" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="10" spans="1:9">
       <c r="A10" t="s">
@@ -6430,6 +6470,9 @@
       <c r="G10" s="1">
         <v>45.56</v>
       </c>
+      <c r="H10" t="s">
+        <v>17</v>
+      </c>
       <c r="I10" s="1"/>
     </row>
     <row r="11" spans="1:9">
@@ -6454,6 +6497,9 @@
       <c r="G11" s="1">
         <v>58.32</v>
       </c>
+      <c r="H11" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="12" spans="1:9">
       <c r="A12" t="s">
@@ -6477,6 +6523,9 @@
       <c r="G12" s="1">
         <v>43.59</v>
       </c>
+      <c r="H12" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="13" spans="1:9">
       <c r="A13" t="s">
@@ -6500,6 +6549,9 @@
       <c r="G13">
         <v>62.74</v>
       </c>
+      <c r="H13" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="14" spans="1:9">
       <c r="A14" t="s">
@@ -6523,6 +6575,9 @@
       <c r="G14">
         <v>47.03</v>
       </c>
+      <c r="H14" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="15" spans="1:9">
       <c r="A15" t="s">
@@ -6546,6 +6601,9 @@
       <c r="G15">
         <v>38.049999999999997</v>
       </c>
+      <c r="H15" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="16" spans="1:9">
       <c r="A16" t="s">
@@ -6568,6 +6626,9 @@
       </c>
       <c r="G16" s="1">
         <v>51.59</v>
+      </c>
+      <c r="H16" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -6645,7 +6706,7 @@
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B3">
         <v>89.91</v>
@@ -6817,19 +6878,19 @@
         <v>11</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>36</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -7253,7 +7314,7 @@
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B3">
         <v>88.03</v>
@@ -7282,7 +7343,7 @@
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B4">
         <v>87.92</v>
@@ -7369,7 +7430,7 @@
     </row>
     <row r="7" spans="1:9">
       <c r="A7" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B7">
         <v>88.35</v>
@@ -7405,7 +7466,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{126B5B5B-E437-C945-9B34-8DD17CA82909}">
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="22.33203125" customWidth="1"/>
@@ -7426,19 +7487,19 @@
         <v>37</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>41</v>
+        <v>82</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>44</v>
+        <v>83</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>34</v>
@@ -7467,7 +7528,7 @@
         <v>47.18</v>
       </c>
       <c r="H2" t="s">
-        <v>44</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -7493,7 +7554,7 @@
         <v>39.32</v>
       </c>
       <c r="H3" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -7545,7 +7606,7 @@
         <v>40.5</v>
       </c>
       <c r="H5" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -7571,7 +7632,7 @@
         <v>65.28</v>
       </c>
       <c r="H6" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -7597,7 +7658,7 @@
         <v>53.27</v>
       </c>
       <c r="H7" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -7623,7 +7684,7 @@
         <v>44.76</v>
       </c>
       <c r="H8" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -7649,7 +7710,7 @@
         <v>48.52</v>
       </c>
       <c r="H9" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -7675,7 +7736,7 @@
         <v>42.68</v>
       </c>
       <c r="H10" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -7701,7 +7762,7 @@
         <v>58.88</v>
       </c>
       <c r="H11" t="s">
-        <v>44</v>
+        <v>83</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -7727,7 +7788,7 @@
         <v>42.76</v>
       </c>
       <c r="H12" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -7753,7 +7814,7 @@
         <v>63.84</v>
       </c>
       <c r="H13" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -7779,7 +7840,59 @@
         <v>41.62</v>
       </c>
       <c r="H14" t="s">
-        <v>44</v>
+        <v>83</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>44.04</v>
+      </c>
+      <c r="C15">
+        <v>37.79</v>
+      </c>
+      <c r="D15">
+        <v>36.979999999999997</v>
+      </c>
+      <c r="E15" s="1">
+        <v>44.21</v>
+      </c>
+      <c r="F15">
+        <v>38.46</v>
+      </c>
+      <c r="G15">
+        <v>36.520000000000003</v>
+      </c>
+      <c r="H15" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>48.49</v>
+      </c>
+      <c r="C16">
+        <v>48.67</v>
+      </c>
+      <c r="D16">
+        <v>50.29</v>
+      </c>
+      <c r="E16">
+        <v>48.69</v>
+      </c>
+      <c r="F16" s="1">
+        <v>49.85</v>
+      </c>
+      <c r="G16">
+        <v>48.99</v>
+      </c>
+      <c r="H16" t="s">
+        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -7828,7 +7941,7 @@
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B2">
         <v>89.11</v>
@@ -7857,7 +7970,7 @@
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B3">
         <v>89.05</v>
@@ -7886,7 +7999,7 @@
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B4" s="1">
         <v>89.3</v>
@@ -7915,7 +8028,7 @@
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B5">
         <v>88.85</v>
@@ -7944,7 +8057,7 @@
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B6">
         <v>89.04</v>
@@ -7973,7 +8086,7 @@
     </row>
     <row r="7" spans="1:9">
       <c r="A7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B7">
         <v>89.15</v>
@@ -8002,7 +8115,7 @@
     </row>
     <row r="15" spans="1:9">
       <c r="H15" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Cross Diaster Experiment and Baseline Ambilation Experiment
</commit_message>
<xml_diff>
--- a/Ablation experiment.xlsx
+++ b/Ablation experiment.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/haochen/Documents/Development/bright-cmca/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C623E984-AF38-0240-9E36-C4F2E280F6EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FF17398-A4B3-D24F-8B27-8F22C859A7B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4340" yWindow="760" windowWidth="30220" windowHeight="20000" firstSheet="6" activeTab="13" xr2:uid="{79C5FF15-FE7B-B844-917A-3EB10CF0BE82}"/>
+    <workbookView xWindow="4340" yWindow="760" windowWidth="30220" windowHeight="20000" activeTab="2" xr2:uid="{79C5FF15-FE7B-B844-917A-3EB10CF0BE82}"/>
   </bookViews>
   <sheets>
     <sheet name="Overall" sheetId="7" r:id="rId1"/>
@@ -538,15 +538,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>241022</xdr:colOff>
       <xdr:row>9</xdr:row>
-      <xdr:rowOff>181715</xdr:rowOff>
+      <xdr:rowOff>153905</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>99459</xdr:colOff>
+      <xdr:colOff>340481</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>57168</xdr:rowOff>
+      <xdr:rowOff>29358</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -569,7 +569,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="2017189"/>
+          <a:off x="241022" y="1989379"/>
           <a:ext cx="8729897" cy="2730636"/>
         </a:xfrm>
         <a:prstGeom prst="rect">

</xml_diff>